<commit_message>
chore: rimuove file di lock Excel tracciati per errore, aggiorna excel team completato dall'utente
</commit_message>
<xml_diff>
--- a/atleti_non_trovati_pcs_v3.xlsx
+++ b/atleti_non_trovati_pcs_v3.xlsx
@@ -2768,7 +2768,7 @@
     <numFmt numFmtId="176" formatCode="_-&quot;€&quot;* #,##0.00_-;\-&quot;€&quot;* #,##0.00_-;_-&quot;€&quot;* \-??_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="_-&quot;€&quot;* #,##0_-;\-&quot;€&quot;* #,##0_-;_-&quot;€&quot;* \-_-;_-@_-"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2796,13 +2796,6 @@
       <i/>
       <sz val="9"/>
       <color rgb="FF7A7F84"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -3253,28 +3246,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -3283,122 +3279,119 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3407,6 +3400,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -8457,7 +8451,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>449</v>
       </c>
     </row>
@@ -8862,7 +8856,7 @@
       <c r="B22" t="s">
         <v>504</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="5" t="s">
         <v>505</v>
       </c>
       <c r="D22" t="str">
@@ -14920,6 +14914,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C18" r:id="rId1" display="https://www.procyclingstats.com/team/a-r-monex-pro-cyclingteam-2026" tooltip="https://www.procyclingstats.com/team/a-r-monex-pro-cyclingteam-2026"/>
+    <hyperlink ref="C22" r:id="rId2" display="https://www.procyclingstats.com/team/uc-conscio-pedale-del-sile-2026"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>